<commit_message>
Modified column titles in raw datasets for ease of understanding
</commit_message>
<xml_diff>
--- a/data/raw/ellicott_larvae_raw.xlsx
+++ b/data/raw/ellicott_larvae_raw.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aidan\Desktop\RStudio Projects\SCLTS-Deformities\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41ECE422-906F-45F2-8F07-C52106ECBD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2707EB22-2DC8-4D01-BF0A-AF6DF16568E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="960" yWindow="3135" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="62">
   <si>
     <t>pond</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>larval dipnet</t>
-  </si>
-  <si>
-    <t>n/a</t>
   </si>
   <si>
     <t>RESAMPLE; back right fused with 10 toes</t>
@@ -536,6 +533,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="83.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1549,12 +1547,6 @@
       <c r="F24">
         <v>2.46</v>
       </c>
-      <c r="G24" t="s">
-        <v>37</v>
-      </c>
-      <c r="H24" t="s">
-        <v>37</v>
-      </c>
       <c r="I24" t="s">
         <v>19</v>
       </c>
@@ -1571,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="N24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O24" t="s">
         <v>22</v>
@@ -1618,7 +1610,7 @@
         <v>1</v>
       </c>
       <c r="N25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O25" t="s">
         <v>22</v>
@@ -1665,7 +1657,7 @@
         <v>1</v>
       </c>
       <c r="N26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O26" t="s">
         <v>22</v>
@@ -1712,7 +1704,7 @@
         <v>0</v>
       </c>
       <c r="N27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O27" t="s">
         <v>22</v>
@@ -1759,7 +1751,7 @@
         <v>1</v>
       </c>
       <c r="N28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O28" t="s">
         <v>22</v>
@@ -1806,7 +1798,7 @@
         <v>0</v>
       </c>
       <c r="N29" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O29" t="s">
         <v>22</v>
@@ -1853,7 +1845,7 @@
         <v>0</v>
       </c>
       <c r="N30" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O30" t="s">
         <v>22</v>
@@ -1900,7 +1892,7 @@
         <v>1</v>
       </c>
       <c r="N31" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O31" t="s">
         <v>22</v>
@@ -1947,7 +1939,7 @@
         <v>1</v>
       </c>
       <c r="N32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="O32" t="s">
         <v>22</v>
@@ -1994,7 +1986,7 @@
         <v>1</v>
       </c>
       <c r="N33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="O33" t="s">
         <v>22</v>
@@ -2041,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="N34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O34" t="s">
         <v>22</v>
@@ -2088,7 +2080,7 @@
         <v>0</v>
       </c>
       <c r="N35" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O35" t="s">
         <v>22</v>
@@ -2135,7 +2127,7 @@
         <v>0</v>
       </c>
       <c r="N36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O36" t="s">
         <v>22</v>
@@ -2182,7 +2174,7 @@
         <v>1</v>
       </c>
       <c r="N37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="O37" t="s">
         <v>22</v>
@@ -2229,7 +2221,7 @@
         <v>0</v>
       </c>
       <c r="N38" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O38" t="s">
         <v>22</v>
@@ -2276,7 +2268,7 @@
         <v>1</v>
       </c>
       <c r="N39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O39" t="s">
         <v>22</v>
@@ -2323,7 +2315,7 @@
         <v>1</v>
       </c>
       <c r="N40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O40" t="s">
         <v>22</v>
@@ -2370,7 +2362,7 @@
         <v>1</v>
       </c>
       <c r="N41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="O41" t="s">
         <v>22</v>
@@ -2417,7 +2409,7 @@
         <v>1</v>
       </c>
       <c r="N42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O42" t="s">
         <v>22</v>
@@ -2464,7 +2456,7 @@
         <v>1</v>
       </c>
       <c r="N43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O43" t="s">
         <v>22</v>
@@ -2511,7 +2503,7 @@
         <v>1</v>
       </c>
       <c r="N44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O44" t="s">
         <v>22</v>
@@ -2558,7 +2550,7 @@
         <v>1</v>
       </c>
       <c r="N45" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O45" t="s">
         <v>22</v>
@@ -2605,7 +2597,7 @@
         <v>0</v>
       </c>
       <c r="N46" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O46" t="s">
         <v>22</v>
@@ -2652,7 +2644,7 @@
         <v>0</v>
       </c>
       <c r="N47" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O47" t="s">
         <v>22</v>
@@ -2699,7 +2691,7 @@
         <v>1</v>
       </c>
       <c r="N48" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O48" t="s">
         <v>22</v>
@@ -2746,7 +2738,7 @@
         <v>1</v>
       </c>
       <c r="N49" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O49" t="s">
         <v>22</v>
@@ -2793,7 +2785,7 @@
         <v>1</v>
       </c>
       <c r="N50" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O50" t="s">
         <v>22</v>
@@ -2840,7 +2832,7 @@
         <v>1</v>
       </c>
       <c r="N51" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O51" t="s">
         <v>22</v>
@@ -2887,7 +2879,7 @@
         <v>1</v>
       </c>
       <c r="N52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O52" t="s">
         <v>22</v>
@@ -2934,7 +2926,7 @@
         <v>0</v>
       </c>
       <c r="N53" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O53" t="s">
         <v>22</v>
@@ -2981,7 +2973,7 @@
         <v>1</v>
       </c>
       <c r="N54" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O54" t="s">
         <v>22</v>
@@ -3028,7 +3020,7 @@
         <v>1</v>
       </c>
       <c r="N55" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="O55" t="s">
         <v>22</v>
@@ -3075,7 +3067,7 @@
         <v>1</v>
       </c>
       <c r="N56" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O56" t="s">
         <v>22</v>
@@ -3122,7 +3114,7 @@
         <v>1</v>
       </c>
       <c r="N57" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O57" t="s">
         <v>22</v>

</xml_diff>